<commit_message>
- Update app version and minimum server version - Fix Extension Form Re-collection
</commit_message>
<xml_diff>
--- a/app/src/main/res/raw/region_form.xlsx
+++ b/app/src/main/res/raw/region_form.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27795" windowHeight="12195" tabRatio="500" activeTab="2"/>
+    <workbookView windowWidth="27795" windowHeight="12315" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="columns" sheetId="1" r:id="rId1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="79">
   <si>
     <t>group</t>
   </si>
@@ -106,9 +106,6 @@
   </si>
   <si>
     <t xml:space="preserve">1.2. የወላጅ አካባቢ ስም  </t>
-  </si>
-  <si>
-    <t>header2</t>
   </si>
   <si>
     <t>regionLevel</t>
@@ -263,10 +260,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="176" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="178" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="179" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
   <fonts count="21">
     <font>
@@ -291,6 +288,66 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
@@ -300,14 +357,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF006100"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -315,6 +365,14 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
       <color theme="3"/>
       <name val="Arial"/>
       <charset val="134"/>
@@ -323,21 +381,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF3F3F76"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -351,20 +394,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF3F3F3F"/>
@@ -374,15 +403,8 @@
     </font>
     <font>
       <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
-      <color rgb="FF9C6500"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -395,37 +417,12 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="34">
     <fill>
@@ -442,31 +439,157 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFA5A5A5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -478,24 +601,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -508,121 +613,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
+        <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -685,6 +682,24 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="double">
         <color rgb="FF3F3F3F"/>
       </left>
@@ -696,15 +711,6 @@
       </top>
       <bottom style="double">
         <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
       </bottom>
       <diagonal/>
     </border>
@@ -724,11 +730,17 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
       </bottom>
       <diagonal/>
     </border>
@@ -750,30 +762,6 @@
     <border>
       <left/>
       <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
       <top style="thin">
         <color theme="4"/>
       </top>
@@ -782,145 +770,154 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="10" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="15" borderId="12" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="10" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="10" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="177" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -930,7 +927,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -962,10 +959,8 @@
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1301,7 +1296,7 @@
     <col min="10" max="10" width="36.1428571428571" customWidth="1"/>
     <col min="11" max="11" width="30.2" customWidth="1"/>
     <col min="12" max="12" width="21.7238095238095" customWidth="1"/>
-    <col min="13" max="13" width="23.7142857142857" customWidth="1"/>
+    <col min="13" max="13" width="52.1428571428571" customWidth="1"/>
     <col min="14" max="14" width="9.26666666666667" customWidth="1"/>
     <col min="16" max="16" width="16.5714285714286" customWidth="1"/>
     <col min="17" max="17" width="12.7142857142857" customWidth="1"/>
@@ -1353,7 +1348,7 @@
       <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="21" t="s">
+      <c r="P1" s="19" t="s">
         <v>15</v>
       </c>
       <c r="Q1" s="1" t="s">
@@ -1427,25 +1422,25 @@
     </row>
     <row r="4" spans="1:15">
       <c r="A4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" t="s">
         <v>30</v>
-      </c>
-      <c r="D4" t="s">
-        <v>31</v>
       </c>
       <c r="E4" t="s">
         <v>20</v>
       </c>
       <c r="H4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I4" t="s">
         <v>32</v>
       </c>
-      <c r="I4" t="s">
+      <c r="J4" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="K4" s="13" t="s">
         <v>34</v>
-      </c>
-      <c r="K4" s="13" t="s">
-        <v>35</v>
       </c>
       <c r="L4" s="13"/>
       <c r="M4" s="13"/>
@@ -1457,26 +1452,24 @@
       </c>
     </row>
     <row r="5" spans="1:14">
-      <c r="A5" s="1" t="s">
-        <v>30</v>
-      </c>
+      <c r="A5" s="1"/>
       <c r="D5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E5" t="s">
         <v>20</v>
       </c>
       <c r="H5" t="s">
+        <v>36</v>
+      </c>
+      <c r="I5" t="s">
         <v>37</v>
       </c>
-      <c r="I5" t="s">
+      <c r="J5" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="J5" s="2" t="s">
+      <c r="K5" s="13" t="s">
         <v>39</v>
-      </c>
-      <c r="K5" s="13" t="s">
-        <v>40</v>
       </c>
       <c r="L5" s="13"/>
       <c r="M5" s="13"/>
@@ -1485,30 +1478,28 @@
       </c>
     </row>
     <row r="6" spans="1:14">
-      <c r="A6" s="1" t="s">
-        <v>30</v>
-      </c>
+      <c r="A6" s="1"/>
       <c r="D6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E6" t="s">
         <v>20</v>
       </c>
       <c r="H6" t="s">
+        <v>41</v>
+      </c>
+      <c r="I6" t="s">
         <v>42</v>
       </c>
-      <c r="I6" t="s">
+      <c r="J6" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="K6" s="13" t="s">
         <v>43</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="K6" s="13" t="s">
-        <v>44</v>
       </c>
       <c r="L6" s="13"/>
       <c r="M6" s="13" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="N6" t="b">
         <v>1</v>
@@ -1516,30 +1507,30 @@
     </row>
     <row r="7" s="4" customFormat="1" spans="1:15">
       <c r="A7" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="E7" s="4" t="s">
         <v>47</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>48</v>
       </c>
       <c r="F7" s="10"/>
       <c r="G7" s="10"/>
       <c r="H7" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="I7" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="I7" s="4" t="s">
+      <c r="J7" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="J7" s="4" t="s">
+      <c r="K7" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="K7" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="L7" s="15"/>
-      <c r="M7" s="15"/>
+      <c r="L7" s="14"/>
+      <c r="M7" s="14"/>
       <c r="N7" s="4" t="b">
         <v>1</v>
       </c>
@@ -1549,28 +1540,28 @@
     </row>
     <row r="8" s="5" customFormat="1" spans="1:15">
       <c r="A8" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D8" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E8" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="H8" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="H8" s="5" t="s">
+      <c r="I8" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="I8" s="5" t="s">
+      <c r="J8" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="J8" s="16" t="s">
+      <c r="K8" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="K8" s="17" t="s">
-        <v>58</v>
-      </c>
-      <c r="L8" s="17"/>
-      <c r="M8" s="17"/>
+      <c r="L8" s="16"/>
+      <c r="M8" s="16"/>
       <c r="N8" s="5" t="b">
         <v>1</v>
       </c>
@@ -1580,30 +1571,30 @@
     </row>
     <row r="9" s="5" customFormat="1" spans="1:18">
       <c r="A9" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D9" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E9" s="5" t="s">
         <v>59</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>60</v>
       </c>
       <c r="F9" s="11"/>
       <c r="G9" s="11"/>
       <c r="H9" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="J9" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="K9" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="I9" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="J9" s="16" t="s">
-        <v>61</v>
-      </c>
-      <c r="K9" s="17" t="s">
-        <v>62</v>
-      </c>
-      <c r="L9" s="17"/>
-      <c r="M9" s="17"/>
+      <c r="L9" s="16"/>
+      <c r="M9" s="16"/>
       <c r="O9" s="5" t="b">
         <v>1</v>
       </c>
@@ -1613,28 +1604,28 @@
     </row>
     <row r="10" s="6" customFormat="1" spans="1:15">
       <c r="A10" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>20</v>
       </c>
       <c r="H10" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I10" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="I10" s="6" t="s">
+      <c r="J10" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="J10" s="6" t="s">
+      <c r="K10" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="K10" s="18" t="s">
-        <v>67</v>
-      </c>
-      <c r="L10" s="19"/>
-      <c r="M10" s="19"/>
+      <c r="L10" s="17"/>
+      <c r="M10" s="17"/>
       <c r="N10" s="6" t="b">
         <v>1</v>
       </c>
@@ -1656,9 +1647,9 @@
     </row>
     <row r="13" spans="1:13">
       <c r="A13" s="1"/>
-      <c r="K13" s="20"/>
-      <c r="L13" s="20"/>
-      <c r="M13" s="20"/>
+      <c r="K13" s="18"/>
+      <c r="L13" s="18"/>
+      <c r="M13" s="18"/>
     </row>
     <row r="14" spans="1:1">
       <c r="A14" s="1"/>
@@ -1718,7 +1709,7 @@
         <v>3</v>
       </c>
       <c r="B1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C1" t="s">
         <v>7</v>
@@ -1751,41 +1742,41 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" t="s">
         <v>70</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" t="s">
         <v>72</v>
-      </c>
-      <c r="E1" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B2" t="s">
         <v>74</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>75</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="3" t="s">
         <v>77</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="22" spans="9:9">
       <c r="I22" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>

</xml_diff>